<commit_message>
Dividir el formulario Jornada de Vacunacion 2026 en 3 hojas por responsable
Cada pestana (Yesenia, Monica, Cirila) es una copia independiente del
formulario con su nombre precargado en NOMBRES DEL RESPONSABLE.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R7mXj6vg79bgxXbpCBxKYB
</commit_message>
<xml_diff>
--- a/excel/Formulario-Jornada-Vacunacion-2026.xlsx
+++ b/excel/Formulario-Jornada-Vacunacion-2026.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Jornada Vacunacion 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Yesenia" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Mónica" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cirila" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="165" formatCode="0;-0;&quot;—&quot;"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +43,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="000000FF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="000000FF"/>
     </font>
     <font>
@@ -120,14 +127,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -136,7 +143,7 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -145,10 +152,10 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -553,7 +560,1533 @@
           <t>NOMBRES DEL RESPONSABLE:</t>
         </is>
       </c>
-      <c r="G2" s="5" t="n"/>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Yesenia</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>RENIPRESS: 00006126</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>EESS: PS. PRINCIPE DE ASTURIAS</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>RIS: RIS VILLA EL SALVADOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Leyenda: complete FECHA por cada jornada; use "-" o deje en blanco cuando no se aplican dosis de ese indicador. La columna TOTAL DOSIS se calcula automaticamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>FECHA / INDICADORES</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>MENORES DE 1 AÑO
+PENTAV 3RA</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>NIÑOS 1 AÑO</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>NIÑOS 2 - 4 AÑOS</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>5 - 10 AÑOS
+SPR UNICA</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>9 AÑOS
+VPH</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>GESTANTE
+DTPA</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>60 AÑOS A MAS
+NEUMO</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>OTRAS VACUNAS</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL DOSIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>SPR 1RA</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>SPR 2DA</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>SPR 1RA</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>SPR 2DA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="11">
+        <f>SUM(B8:K8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n"/>
+      <c r="B9" s="13" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="13" t="n"/>
+      <c r="F9" s="13" t="n"/>
+      <c r="G9" s="13" t="n"/>
+      <c r="H9" s="13" t="n"/>
+      <c r="I9" s="13" t="n"/>
+      <c r="J9" s="13" t="n"/>
+      <c r="K9" s="13" t="n"/>
+      <c r="L9" s="11">
+        <f>SUM(B9:K9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="13" t="n"/>
+      <c r="C10" s="13" t="n"/>
+      <c r="D10" s="13" t="n"/>
+      <c r="E10" s="13" t="n"/>
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="13" t="n"/>
+      <c r="H10" s="13" t="n"/>
+      <c r="I10" s="13" t="n"/>
+      <c r="J10" s="13" t="n"/>
+      <c r="K10" s="13" t="n"/>
+      <c r="L10" s="11">
+        <f>SUM(B10:K10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="13" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="13" t="n"/>
+      <c r="F11" s="13" t="n"/>
+      <c r="G11" s="13" t="n"/>
+      <c r="H11" s="13" t="n"/>
+      <c r="I11" s="13" t="n"/>
+      <c r="J11" s="13" t="n"/>
+      <c r="K11" s="13" t="n"/>
+      <c r="L11" s="11">
+        <f>SUM(B11:K11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="13" t="n"/>
+      <c r="I12" s="13" t="n"/>
+      <c r="J12" s="13" t="n"/>
+      <c r="K12" s="13" t="n"/>
+      <c r="L12" s="11">
+        <f>SUM(B12:K12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+      <c r="H13" s="13" t="n"/>
+      <c r="I13" s="13" t="n"/>
+      <c r="J13" s="13" t="n"/>
+      <c r="K13" s="13" t="n"/>
+      <c r="L13" s="11">
+        <f>SUM(B13:K13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="13" t="n"/>
+      <c r="I14" s="13" t="n"/>
+      <c r="J14" s="13" t="n"/>
+      <c r="K14" s="13" t="n"/>
+      <c r="L14" s="11">
+        <f>SUM(B14:K14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="13" t="n"/>
+      <c r="C15" s="13" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="13" t="n"/>
+      <c r="G15" s="13" t="n"/>
+      <c r="H15" s="13" t="n"/>
+      <c r="I15" s="13" t="n"/>
+      <c r="J15" s="13" t="n"/>
+      <c r="K15" s="13" t="n"/>
+      <c r="L15" s="11">
+        <f>SUM(B15:K15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="13" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="13" t="n"/>
+      <c r="I16" s="13" t="n"/>
+      <c r="J16" s="13" t="n"/>
+      <c r="K16" s="13" t="n"/>
+      <c r="L16" s="11">
+        <f>SUM(B16:K16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="13" t="n"/>
+      <c r="F17" s="13" t="n"/>
+      <c r="G17" s="13" t="n"/>
+      <c r="H17" s="13" t="n"/>
+      <c r="I17" s="13" t="n"/>
+      <c r="J17" s="13" t="n"/>
+      <c r="K17" s="13" t="n"/>
+      <c r="L17" s="11">
+        <f>SUM(B17:K17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="13" t="n"/>
+      <c r="I18" s="13" t="n"/>
+      <c r="J18" s="13" t="n"/>
+      <c r="K18" s="13" t="n"/>
+      <c r="L18" s="11">
+        <f>SUM(B18:K18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="n"/>
+      <c r="K19" s="13" t="n"/>
+      <c r="L19" s="11">
+        <f>SUM(B19:K19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="13" t="n"/>
+      <c r="D20" s="13" t="n"/>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="13" t="n"/>
+      <c r="G20" s="13" t="n"/>
+      <c r="H20" s="13" t="n"/>
+      <c r="I20" s="13" t="n"/>
+      <c r="J20" s="13" t="n"/>
+      <c r="K20" s="13" t="n"/>
+      <c r="L20" s="11">
+        <f>SUM(B20:K20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n"/>
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="13" t="n"/>
+      <c r="D21" s="13" t="n"/>
+      <c r="E21" s="13" t="n"/>
+      <c r="F21" s="13" t="n"/>
+      <c r="G21" s="13" t="n"/>
+      <c r="H21" s="13" t="n"/>
+      <c r="I21" s="13" t="n"/>
+      <c r="J21" s="13" t="n"/>
+      <c r="K21" s="13" t="n"/>
+      <c r="L21" s="11">
+        <f>SUM(B21:K21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n"/>
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="n"/>
+      <c r="D22" s="13" t="n"/>
+      <c r="E22" s="13" t="n"/>
+      <c r="F22" s="13" t="n"/>
+      <c r="G22" s="13" t="n"/>
+      <c r="H22" s="13" t="n"/>
+      <c r="I22" s="13" t="n"/>
+      <c r="J22" s="13" t="n"/>
+      <c r="K22" s="13" t="n"/>
+      <c r="L22" s="11">
+        <f>SUM(B22:K22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n"/>
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="n"/>
+      <c r="D23" s="13" t="n"/>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="13" t="n"/>
+      <c r="G23" s="13" t="n"/>
+      <c r="H23" s="13" t="n"/>
+      <c r="I23" s="13" t="n"/>
+      <c r="J23" s="13" t="n"/>
+      <c r="K23" s="13" t="n"/>
+      <c r="L23" s="11">
+        <f>SUM(B23:K23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n"/>
+      <c r="B24" s="13" t="n"/>
+      <c r="C24" s="13" t="n"/>
+      <c r="D24" s="13" t="n"/>
+      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="13" t="n"/>
+      <c r="G24" s="13" t="n"/>
+      <c r="H24" s="13" t="n"/>
+      <c r="I24" s="13" t="n"/>
+      <c r="J24" s="13" t="n"/>
+      <c r="K24" s="13" t="n"/>
+      <c r="L24" s="11">
+        <f>SUM(B24:K24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n"/>
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="13" t="n"/>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="13" t="n"/>
+      <c r="F25" s="13" t="n"/>
+      <c r="G25" s="13" t="n"/>
+      <c r="H25" s="13" t="n"/>
+      <c r="I25" s="13" t="n"/>
+      <c r="J25" s="13" t="n"/>
+      <c r="K25" s="13" t="n"/>
+      <c r="L25" s="11">
+        <f>SUM(B25:K25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n"/>
+      <c r="B26" s="13" t="n"/>
+      <c r="C26" s="13" t="n"/>
+      <c r="D26" s="13" t="n"/>
+      <c r="E26" s="13" t="n"/>
+      <c r="F26" s="13" t="n"/>
+      <c r="G26" s="13" t="n"/>
+      <c r="H26" s="13" t="n"/>
+      <c r="I26" s="13" t="n"/>
+      <c r="J26" s="13" t="n"/>
+      <c r="K26" s="13" t="n"/>
+      <c r="L26" s="11">
+        <f>SUM(B26:K26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n"/>
+      <c r="B27" s="13" t="n"/>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="13" t="n"/>
+      <c r="E27" s="13" t="n"/>
+      <c r="F27" s="13" t="n"/>
+      <c r="G27" s="13" t="n"/>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="n"/>
+      <c r="J27" s="13" t="n"/>
+      <c r="K27" s="13" t="n"/>
+      <c r="L27" s="11">
+        <f>SUM(B27:K27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n"/>
+      <c r="B28" s="13" t="n"/>
+      <c r="C28" s="13" t="n"/>
+      <c r="D28" s="13" t="n"/>
+      <c r="E28" s="13" t="n"/>
+      <c r="F28" s="13" t="n"/>
+      <c r="G28" s="13" t="n"/>
+      <c r="H28" s="13" t="n"/>
+      <c r="I28" s="13" t="n"/>
+      <c r="J28" s="13" t="n"/>
+      <c r="K28" s="13" t="n"/>
+      <c r="L28" s="11">
+        <f>SUM(B28:K28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n"/>
+      <c r="B29" s="13" t="n"/>
+      <c r="C29" s="13" t="n"/>
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="13" t="n"/>
+      <c r="F29" s="13" t="n"/>
+      <c r="G29" s="13" t="n"/>
+      <c r="H29" s="13" t="n"/>
+      <c r="I29" s="13" t="n"/>
+      <c r="J29" s="13" t="n"/>
+      <c r="K29" s="13" t="n"/>
+      <c r="L29" s="11">
+        <f>SUM(B29:K29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n"/>
+      <c r="B30" s="13" t="n"/>
+      <c r="C30" s="13" t="n"/>
+      <c r="D30" s="13" t="n"/>
+      <c r="E30" s="13" t="n"/>
+      <c r="F30" s="13" t="n"/>
+      <c r="G30" s="13" t="n"/>
+      <c r="H30" s="13" t="n"/>
+      <c r="I30" s="13" t="n"/>
+      <c r="J30" s="13" t="n"/>
+      <c r="K30" s="13" t="n"/>
+      <c r="L30" s="11">
+        <f>SUM(B30:K30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n"/>
+      <c r="B31" s="13" t="n"/>
+      <c r="C31" s="13" t="n"/>
+      <c r="D31" s="13" t="n"/>
+      <c r="E31" s="13" t="n"/>
+      <c r="F31" s="13" t="n"/>
+      <c r="G31" s="13" t="n"/>
+      <c r="H31" s="13" t="n"/>
+      <c r="I31" s="13" t="n"/>
+      <c r="J31" s="13" t="n"/>
+      <c r="K31" s="13" t="n"/>
+      <c r="L31" s="11">
+        <f>SUM(B31:K31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n"/>
+      <c r="B32" s="13" t="n"/>
+      <c r="C32" s="13" t="n"/>
+      <c r="D32" s="13" t="n"/>
+      <c r="E32" s="13" t="n"/>
+      <c r="F32" s="13" t="n"/>
+      <c r="G32" s="13" t="n"/>
+      <c r="H32" s="13" t="n"/>
+      <c r="I32" s="13" t="n"/>
+      <c r="J32" s="13" t="n"/>
+      <c r="K32" s="13" t="n"/>
+      <c r="L32" s="11">
+        <f>SUM(B32:K32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n"/>
+      <c r="B33" s="13" t="n"/>
+      <c r="C33" s="13" t="n"/>
+      <c r="D33" s="13" t="n"/>
+      <c r="E33" s="13" t="n"/>
+      <c r="F33" s="13" t="n"/>
+      <c r="G33" s="13" t="n"/>
+      <c r="H33" s="13" t="n"/>
+      <c r="I33" s="13" t="n"/>
+      <c r="J33" s="13" t="n"/>
+      <c r="K33" s="13" t="n"/>
+      <c r="L33" s="11">
+        <f>SUM(B33:K33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="n"/>
+      <c r="B34" s="13" t="n"/>
+      <c r="C34" s="13" t="n"/>
+      <c r="D34" s="13" t="n"/>
+      <c r="E34" s="13" t="n"/>
+      <c r="F34" s="13" t="n"/>
+      <c r="G34" s="13" t="n"/>
+      <c r="H34" s="13" t="n"/>
+      <c r="I34" s="13" t="n"/>
+      <c r="J34" s="13" t="n"/>
+      <c r="K34" s="13" t="n"/>
+      <c r="L34" s="11">
+        <f>SUM(B34:K34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n"/>
+      <c r="B35" s="13" t="n"/>
+      <c r="C35" s="13" t="n"/>
+      <c r="D35" s="13" t="n"/>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="13" t="n"/>
+      <c r="G35" s="13" t="n"/>
+      <c r="H35" s="13" t="n"/>
+      <c r="I35" s="13" t="n"/>
+      <c r="J35" s="13" t="n"/>
+      <c r="K35" s="13" t="n"/>
+      <c r="L35" s="11">
+        <f>SUM(B35:K35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n"/>
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="13" t="n"/>
+      <c r="D36" s="13" t="n"/>
+      <c r="E36" s="13" t="n"/>
+      <c r="F36" s="13" t="n"/>
+      <c r="G36" s="13" t="n"/>
+      <c r="H36" s="13" t="n"/>
+      <c r="I36" s="13" t="n"/>
+      <c r="J36" s="13" t="n"/>
+      <c r="K36" s="13" t="n"/>
+      <c r="L36" s="11">
+        <f>SUM(B36:K36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n"/>
+      <c r="B37" s="13" t="n"/>
+      <c r="C37" s="13" t="n"/>
+      <c r="D37" s="13" t="n"/>
+      <c r="E37" s="13" t="n"/>
+      <c r="F37" s="13" t="n"/>
+      <c r="G37" s="13" t="n"/>
+      <c r="H37" s="13" t="n"/>
+      <c r="I37" s="13" t="n"/>
+      <c r="J37" s="13" t="n"/>
+      <c r="K37" s="13" t="n"/>
+      <c r="L37" s="11">
+        <f>SUM(B37:K37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B38" s="15">
+        <f>SUM(B8:B37)</f>
+        <v/>
+      </c>
+      <c r="C38" s="15">
+        <f>SUM(C8:C37)</f>
+        <v/>
+      </c>
+      <c r="D38" s="15">
+        <f>SUM(D8:D37)</f>
+        <v/>
+      </c>
+      <c r="E38" s="15">
+        <f>SUM(E8:E37)</f>
+        <v/>
+      </c>
+      <c r="F38" s="15">
+        <f>SUM(F8:F37)</f>
+        <v/>
+      </c>
+      <c r="G38" s="15">
+        <f>SUM(G8:G37)</f>
+        <v/>
+      </c>
+      <c r="H38" s="15">
+        <f>SUM(H8:H37)</f>
+        <v/>
+      </c>
+      <c r="I38" s="15">
+        <f>SUM(I8:I37)</f>
+        <v/>
+      </c>
+      <c r="J38" s="15">
+        <f>SUM(J8:J37)</f>
+        <v/>
+      </c>
+      <c r="K38" s="15">
+        <f>SUM(K8:K37)</f>
+        <v/>
+      </c>
+      <c r="L38" s="15">
+        <f>SUM(L8:L37)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="G2:L2"/>
+    <mergeCell ref="I3:L3"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="K6:K7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>JORNADA DE VACUNACION 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>FECHA:</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>NOMBRES DEL RESPONSABLE:</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Mónica</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>RENIPRESS: 00006126</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>EESS: PS. PRINCIPE DE ASTURIAS</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>RIS: RIS VILLA EL SALVADOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Leyenda: complete FECHA por cada jornada; use "-" o deje en blanco cuando no se aplican dosis de ese indicador. La columna TOTAL DOSIS se calcula automaticamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>FECHA / INDICADORES</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>MENORES DE 1 AÑO
+PENTAV 3RA</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>NIÑOS 1 AÑO</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>NIÑOS 2 - 4 AÑOS</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>5 - 10 AÑOS
+SPR UNICA</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>9 AÑOS
+VPH</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>GESTANTE
+DTPA</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>60 AÑOS A MAS
+NEUMO</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>OTRAS VACUNAS</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL DOSIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>SPR 1RA</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>SPR 2DA</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>SPR 1RA</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>SPR 2DA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="11">
+        <f>SUM(B8:K8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n"/>
+      <c r="B9" s="13" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="13" t="n"/>
+      <c r="F9" s="13" t="n"/>
+      <c r="G9" s="13" t="n"/>
+      <c r="H9" s="13" t="n"/>
+      <c r="I9" s="13" t="n"/>
+      <c r="J9" s="13" t="n"/>
+      <c r="K9" s="13" t="n"/>
+      <c r="L9" s="11">
+        <f>SUM(B9:K9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="13" t="n"/>
+      <c r="C10" s="13" t="n"/>
+      <c r="D10" s="13" t="n"/>
+      <c r="E10" s="13" t="n"/>
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="13" t="n"/>
+      <c r="H10" s="13" t="n"/>
+      <c r="I10" s="13" t="n"/>
+      <c r="J10" s="13" t="n"/>
+      <c r="K10" s="13" t="n"/>
+      <c r="L10" s="11">
+        <f>SUM(B10:K10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="13" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="13" t="n"/>
+      <c r="F11" s="13" t="n"/>
+      <c r="G11" s="13" t="n"/>
+      <c r="H11" s="13" t="n"/>
+      <c r="I11" s="13" t="n"/>
+      <c r="J11" s="13" t="n"/>
+      <c r="K11" s="13" t="n"/>
+      <c r="L11" s="11">
+        <f>SUM(B11:K11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="13" t="n"/>
+      <c r="I12" s="13" t="n"/>
+      <c r="J12" s="13" t="n"/>
+      <c r="K12" s="13" t="n"/>
+      <c r="L12" s="11">
+        <f>SUM(B12:K12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+      <c r="H13" s="13" t="n"/>
+      <c r="I13" s="13" t="n"/>
+      <c r="J13" s="13" t="n"/>
+      <c r="K13" s="13" t="n"/>
+      <c r="L13" s="11">
+        <f>SUM(B13:K13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="13" t="n"/>
+      <c r="I14" s="13" t="n"/>
+      <c r="J14" s="13" t="n"/>
+      <c r="K14" s="13" t="n"/>
+      <c r="L14" s="11">
+        <f>SUM(B14:K14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="13" t="n"/>
+      <c r="C15" s="13" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="13" t="n"/>
+      <c r="G15" s="13" t="n"/>
+      <c r="H15" s="13" t="n"/>
+      <c r="I15" s="13" t="n"/>
+      <c r="J15" s="13" t="n"/>
+      <c r="K15" s="13" t="n"/>
+      <c r="L15" s="11">
+        <f>SUM(B15:K15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="13" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="13" t="n"/>
+      <c r="I16" s="13" t="n"/>
+      <c r="J16" s="13" t="n"/>
+      <c r="K16" s="13" t="n"/>
+      <c r="L16" s="11">
+        <f>SUM(B16:K16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="13" t="n"/>
+      <c r="F17" s="13" t="n"/>
+      <c r="G17" s="13" t="n"/>
+      <c r="H17" s="13" t="n"/>
+      <c r="I17" s="13" t="n"/>
+      <c r="J17" s="13" t="n"/>
+      <c r="K17" s="13" t="n"/>
+      <c r="L17" s="11">
+        <f>SUM(B17:K17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="13" t="n"/>
+      <c r="I18" s="13" t="n"/>
+      <c r="J18" s="13" t="n"/>
+      <c r="K18" s="13" t="n"/>
+      <c r="L18" s="11">
+        <f>SUM(B18:K18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="n"/>
+      <c r="K19" s="13" t="n"/>
+      <c r="L19" s="11">
+        <f>SUM(B19:K19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="13" t="n"/>
+      <c r="D20" s="13" t="n"/>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="13" t="n"/>
+      <c r="G20" s="13" t="n"/>
+      <c r="H20" s="13" t="n"/>
+      <c r="I20" s="13" t="n"/>
+      <c r="J20" s="13" t="n"/>
+      <c r="K20" s="13" t="n"/>
+      <c r="L20" s="11">
+        <f>SUM(B20:K20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n"/>
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="13" t="n"/>
+      <c r="D21" s="13" t="n"/>
+      <c r="E21" s="13" t="n"/>
+      <c r="F21" s="13" t="n"/>
+      <c r="G21" s="13" t="n"/>
+      <c r="H21" s="13" t="n"/>
+      <c r="I21" s="13" t="n"/>
+      <c r="J21" s="13" t="n"/>
+      <c r="K21" s="13" t="n"/>
+      <c r="L21" s="11">
+        <f>SUM(B21:K21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n"/>
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="n"/>
+      <c r="D22" s="13" t="n"/>
+      <c r="E22" s="13" t="n"/>
+      <c r="F22" s="13" t="n"/>
+      <c r="G22" s="13" t="n"/>
+      <c r="H22" s="13" t="n"/>
+      <c r="I22" s="13" t="n"/>
+      <c r="J22" s="13" t="n"/>
+      <c r="K22" s="13" t="n"/>
+      <c r="L22" s="11">
+        <f>SUM(B22:K22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n"/>
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="n"/>
+      <c r="D23" s="13" t="n"/>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="13" t="n"/>
+      <c r="G23" s="13" t="n"/>
+      <c r="H23" s="13" t="n"/>
+      <c r="I23" s="13" t="n"/>
+      <c r="J23" s="13" t="n"/>
+      <c r="K23" s="13" t="n"/>
+      <c r="L23" s="11">
+        <f>SUM(B23:K23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n"/>
+      <c r="B24" s="13" t="n"/>
+      <c r="C24" s="13" t="n"/>
+      <c r="D24" s="13" t="n"/>
+      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="13" t="n"/>
+      <c r="G24" s="13" t="n"/>
+      <c r="H24" s="13" t="n"/>
+      <c r="I24" s="13" t="n"/>
+      <c r="J24" s="13" t="n"/>
+      <c r="K24" s="13" t="n"/>
+      <c r="L24" s="11">
+        <f>SUM(B24:K24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n"/>
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="13" t="n"/>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="13" t="n"/>
+      <c r="F25" s="13" t="n"/>
+      <c r="G25" s="13" t="n"/>
+      <c r="H25" s="13" t="n"/>
+      <c r="I25" s="13" t="n"/>
+      <c r="J25" s="13" t="n"/>
+      <c r="K25" s="13" t="n"/>
+      <c r="L25" s="11">
+        <f>SUM(B25:K25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n"/>
+      <c r="B26" s="13" t="n"/>
+      <c r="C26" s="13" t="n"/>
+      <c r="D26" s="13" t="n"/>
+      <c r="E26" s="13" t="n"/>
+      <c r="F26" s="13" t="n"/>
+      <c r="G26" s="13" t="n"/>
+      <c r="H26" s="13" t="n"/>
+      <c r="I26" s="13" t="n"/>
+      <c r="J26" s="13" t="n"/>
+      <c r="K26" s="13" t="n"/>
+      <c r="L26" s="11">
+        <f>SUM(B26:K26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n"/>
+      <c r="B27" s="13" t="n"/>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="13" t="n"/>
+      <c r="E27" s="13" t="n"/>
+      <c r="F27" s="13" t="n"/>
+      <c r="G27" s="13" t="n"/>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="n"/>
+      <c r="J27" s="13" t="n"/>
+      <c r="K27" s="13" t="n"/>
+      <c r="L27" s="11">
+        <f>SUM(B27:K27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n"/>
+      <c r="B28" s="13" t="n"/>
+      <c r="C28" s="13" t="n"/>
+      <c r="D28" s="13" t="n"/>
+      <c r="E28" s="13" t="n"/>
+      <c r="F28" s="13" t="n"/>
+      <c r="G28" s="13" t="n"/>
+      <c r="H28" s="13" t="n"/>
+      <c r="I28" s="13" t="n"/>
+      <c r="J28" s="13" t="n"/>
+      <c r="K28" s="13" t="n"/>
+      <c r="L28" s="11">
+        <f>SUM(B28:K28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n"/>
+      <c r="B29" s="13" t="n"/>
+      <c r="C29" s="13" t="n"/>
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="13" t="n"/>
+      <c r="F29" s="13" t="n"/>
+      <c r="G29" s="13" t="n"/>
+      <c r="H29" s="13" t="n"/>
+      <c r="I29" s="13" t="n"/>
+      <c r="J29" s="13" t="n"/>
+      <c r="K29" s="13" t="n"/>
+      <c r="L29" s="11">
+        <f>SUM(B29:K29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n"/>
+      <c r="B30" s="13" t="n"/>
+      <c r="C30" s="13" t="n"/>
+      <c r="D30" s="13" t="n"/>
+      <c r="E30" s="13" t="n"/>
+      <c r="F30" s="13" t="n"/>
+      <c r="G30" s="13" t="n"/>
+      <c r="H30" s="13" t="n"/>
+      <c r="I30" s="13" t="n"/>
+      <c r="J30" s="13" t="n"/>
+      <c r="K30" s="13" t="n"/>
+      <c r="L30" s="11">
+        <f>SUM(B30:K30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n"/>
+      <c r="B31" s="13" t="n"/>
+      <c r="C31" s="13" t="n"/>
+      <c r="D31" s="13" t="n"/>
+      <c r="E31" s="13" t="n"/>
+      <c r="F31" s="13" t="n"/>
+      <c r="G31" s="13" t="n"/>
+      <c r="H31" s="13" t="n"/>
+      <c r="I31" s="13" t="n"/>
+      <c r="J31" s="13" t="n"/>
+      <c r="K31" s="13" t="n"/>
+      <c r="L31" s="11">
+        <f>SUM(B31:K31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n"/>
+      <c r="B32" s="13" t="n"/>
+      <c r="C32" s="13" t="n"/>
+      <c r="D32" s="13" t="n"/>
+      <c r="E32" s="13" t="n"/>
+      <c r="F32" s="13" t="n"/>
+      <c r="G32" s="13" t="n"/>
+      <c r="H32" s="13" t="n"/>
+      <c r="I32" s="13" t="n"/>
+      <c r="J32" s="13" t="n"/>
+      <c r="K32" s="13" t="n"/>
+      <c r="L32" s="11">
+        <f>SUM(B32:K32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n"/>
+      <c r="B33" s="13" t="n"/>
+      <c r="C33" s="13" t="n"/>
+      <c r="D33" s="13" t="n"/>
+      <c r="E33" s="13" t="n"/>
+      <c r="F33" s="13" t="n"/>
+      <c r="G33" s="13" t="n"/>
+      <c r="H33" s="13" t="n"/>
+      <c r="I33" s="13" t="n"/>
+      <c r="J33" s="13" t="n"/>
+      <c r="K33" s="13" t="n"/>
+      <c r="L33" s="11">
+        <f>SUM(B33:K33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="n"/>
+      <c r="B34" s="13" t="n"/>
+      <c r="C34" s="13" t="n"/>
+      <c r="D34" s="13" t="n"/>
+      <c r="E34" s="13" t="n"/>
+      <c r="F34" s="13" t="n"/>
+      <c r="G34" s="13" t="n"/>
+      <c r="H34" s="13" t="n"/>
+      <c r="I34" s="13" t="n"/>
+      <c r="J34" s="13" t="n"/>
+      <c r="K34" s="13" t="n"/>
+      <c r="L34" s="11">
+        <f>SUM(B34:K34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n"/>
+      <c r="B35" s="13" t="n"/>
+      <c r="C35" s="13" t="n"/>
+      <c r="D35" s="13" t="n"/>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="13" t="n"/>
+      <c r="G35" s="13" t="n"/>
+      <c r="H35" s="13" t="n"/>
+      <c r="I35" s="13" t="n"/>
+      <c r="J35" s="13" t="n"/>
+      <c r="K35" s="13" t="n"/>
+      <c r="L35" s="11">
+        <f>SUM(B35:K35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n"/>
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="13" t="n"/>
+      <c r="D36" s="13" t="n"/>
+      <c r="E36" s="13" t="n"/>
+      <c r="F36" s="13" t="n"/>
+      <c r="G36" s="13" t="n"/>
+      <c r="H36" s="13" t="n"/>
+      <c r="I36" s="13" t="n"/>
+      <c r="J36" s="13" t="n"/>
+      <c r="K36" s="13" t="n"/>
+      <c r="L36" s="11">
+        <f>SUM(B36:K36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n"/>
+      <c r="B37" s="13" t="n"/>
+      <c r="C37" s="13" t="n"/>
+      <c r="D37" s="13" t="n"/>
+      <c r="E37" s="13" t="n"/>
+      <c r="F37" s="13" t="n"/>
+      <c r="G37" s="13" t="n"/>
+      <c r="H37" s="13" t="n"/>
+      <c r="I37" s="13" t="n"/>
+      <c r="J37" s="13" t="n"/>
+      <c r="K37" s="13" t="n"/>
+      <c r="L37" s="11">
+        <f>SUM(B37:K37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B38" s="15">
+        <f>SUM(B8:B37)</f>
+        <v/>
+      </c>
+      <c r="C38" s="15">
+        <f>SUM(C8:C37)</f>
+        <v/>
+      </c>
+      <c r="D38" s="15">
+        <f>SUM(D8:D37)</f>
+        <v/>
+      </c>
+      <c r="E38" s="15">
+        <f>SUM(E8:E37)</f>
+        <v/>
+      </c>
+      <c r="F38" s="15">
+        <f>SUM(F8:F37)</f>
+        <v/>
+      </c>
+      <c r="G38" s="15">
+        <f>SUM(G8:G37)</f>
+        <v/>
+      </c>
+      <c r="H38" s="15">
+        <f>SUM(H8:H37)</f>
+        <v/>
+      </c>
+      <c r="I38" s="15">
+        <f>SUM(I8:I37)</f>
+        <v/>
+      </c>
+      <c r="J38" s="15">
+        <f>SUM(J8:J37)</f>
+        <v/>
+      </c>
+      <c r="K38" s="15">
+        <f>SUM(K8:K37)</f>
+        <v/>
+      </c>
+      <c r="L38" s="15">
+        <f>SUM(L8:L37)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="G2:L2"/>
+    <mergeCell ref="I3:L3"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="K6:K7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>JORNADA DE VACUNACION 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>FECHA:</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>NOMBRES DEL RESPONSABLE:</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Cirila</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Agregar hoja Resumen con totales consolidados por formula
La nueva pestana Resumen suma automaticamente (referencias cruzadas
='Hoja'!celda) el TOTAL GENERAL de cada responsable (Yesenia, Monica,
Cirila) para que no haya que sumarlos a mano antes de digitar el dato
en el sistema.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R7mXj6vg79bgxXbpCBxKYB
</commit_message>
<xml_diff>
--- a/excel/Formulario-Jornada-Vacunacion-2026.xlsx
+++ b/excel/Formulario-Jornada-Vacunacion-2026.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Yesenia" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Mónica" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cirila" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Yesenia" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Mónica" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cirila" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -89,7 +90,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -111,11 +112,88 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -158,6 +236,15 @@
     <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -523,10 +610,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -541,738 +628,289 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>JORNADA DE VACUNACION 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>FECHA:</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>NOMBRES DEL RESPONSABLE:</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>RESUMEN CONSOLIDADO - JORNADA DE VACUNACION 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>RESPONSABLE</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>PENTAV 3RA</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>SPR 1RA (1a)</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>SPR 2DA (1a)</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>SPR 1RA (2-4a)</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>SPR 2DA (2-4a)</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>SPR UNICA</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>VPH</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>DTPA</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>NEUMO</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>OTRAS VACUNAS</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL DOSIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Yesenia</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>RENIPRESS: 00006126</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>EESS: PS. PRINCIPE DE ASTURIAS</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>RIS: RIS VILLA EL SALVADOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Leyenda: complete FECHA por cada jornada; use "-" o deje en blanco cuando no se aplican dosis de ese indicador. La columna TOTAL DOSIS se calcula automaticamente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>FECHA / INDICADORES</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>MENORES DE 1 AÑO
-PENTAV 3RA</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>NIÑOS 1 AÑO</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>NIÑOS 2 - 4 AÑOS</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>5 - 10 AÑOS
-SPR UNICA</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>9 AÑOS
-VPH</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr">
-        <is>
-          <t>GESTANTE
-DTPA</t>
-        </is>
-      </c>
-      <c r="J6" s="7" t="inlineStr">
-        <is>
-          <t>60 AÑOS A MAS
-NEUMO</t>
-        </is>
-      </c>
-      <c r="K6" s="7" t="inlineStr">
-        <is>
-          <t>OTRAS VACUNAS</t>
-        </is>
-      </c>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL DOSIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>SPR 1RA</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>SPR 2DA</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>SPR 1RA</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>SPR 2DA</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="n">
-        <v>46027</v>
-      </c>
-      <c r="B8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="11">
-        <f>SUM(B8:K8)</f>
+      <c r="B4" s="13">
+        <f>'Yesenia'!B38</f>
+        <v/>
+      </c>
+      <c r="C4" s="13">
+        <f>'Yesenia'!C38</f>
+        <v/>
+      </c>
+      <c r="D4" s="13">
+        <f>'Yesenia'!D38</f>
+        <v/>
+      </c>
+      <c r="E4" s="13">
+        <f>'Yesenia'!E38</f>
+        <v/>
+      </c>
+      <c r="F4" s="13">
+        <f>'Yesenia'!F38</f>
+        <v/>
+      </c>
+      <c r="G4" s="13">
+        <f>'Yesenia'!G38</f>
+        <v/>
+      </c>
+      <c r="H4" s="13">
+        <f>'Yesenia'!H38</f>
+        <v/>
+      </c>
+      <c r="I4" s="13">
+        <f>'Yesenia'!I38</f>
+        <v/>
+      </c>
+      <c r="J4" s="13">
+        <f>'Yesenia'!J38</f>
+        <v/>
+      </c>
+      <c r="K4" s="13">
+        <f>'Yesenia'!K38</f>
+        <v/>
+      </c>
+      <c r="L4" s="13">
+        <f>'Yesenia'!L38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Mónica</t>
+        </is>
+      </c>
+      <c r="B5" s="13">
+        <f>'Mónica'!B38</f>
+        <v/>
+      </c>
+      <c r="C5" s="13">
+        <f>'Mónica'!C38</f>
+        <v/>
+      </c>
+      <c r="D5" s="13">
+        <f>'Mónica'!D38</f>
+        <v/>
+      </c>
+      <c r="E5" s="13">
+        <f>'Mónica'!E38</f>
+        <v/>
+      </c>
+      <c r="F5" s="13">
+        <f>'Mónica'!F38</f>
+        <v/>
+      </c>
+      <c r="G5" s="13">
+        <f>'Mónica'!G38</f>
+        <v/>
+      </c>
+      <c r="H5" s="13">
+        <f>'Mónica'!H38</f>
+        <v/>
+      </c>
+      <c r="I5" s="13">
+        <f>'Mónica'!I38</f>
+        <v/>
+      </c>
+      <c r="J5" s="13">
+        <f>'Mónica'!J38</f>
+        <v/>
+      </c>
+      <c r="K5" s="13">
+        <f>'Mónica'!K38</f>
+        <v/>
+      </c>
+      <c r="L5" s="13">
+        <f>'Mónica'!L38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Cirila</t>
+        </is>
+      </c>
+      <c r="B6" s="13">
+        <f>'Cirila'!B38</f>
+        <v/>
+      </c>
+      <c r="C6" s="13">
+        <f>'Cirila'!C38</f>
+        <v/>
+      </c>
+      <c r="D6" s="13">
+        <f>'Cirila'!D38</f>
+        <v/>
+      </c>
+      <c r="E6" s="13">
+        <f>'Cirila'!E38</f>
+        <v/>
+      </c>
+      <c r="F6" s="13">
+        <f>'Cirila'!F38</f>
+        <v/>
+      </c>
+      <c r="G6" s="13">
+        <f>'Cirila'!G38</f>
+        <v/>
+      </c>
+      <c r="H6" s="13">
+        <f>'Cirila'!H38</f>
+        <v/>
+      </c>
+      <c r="I6" s="13">
+        <f>'Cirila'!I38</f>
+        <v/>
+      </c>
+      <c r="J6" s="13">
+        <f>'Cirila'!J38</f>
+        <v/>
+      </c>
+      <c r="K6" s="13">
+        <f>'Cirila'!K38</f>
+        <v/>
+      </c>
+      <c r="L6" s="13">
+        <f>'Cirila'!L38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B7" s="15">
+        <f>SUM(B4:B6)</f>
+        <v/>
+      </c>
+      <c r="C7" s="15">
+        <f>SUM(C4:C6)</f>
+        <v/>
+      </c>
+      <c r="D7" s="15">
+        <f>SUM(D4:D6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="15">
+        <f>SUM(E4:E6)</f>
+        <v/>
+      </c>
+      <c r="F7" s="15">
+        <f>SUM(F4:F6)</f>
+        <v/>
+      </c>
+      <c r="G7" s="15">
+        <f>SUM(G4:G6)</f>
+        <v/>
+      </c>
+      <c r="H7" s="15">
+        <f>SUM(H4:H6)</f>
+        <v/>
+      </c>
+      <c r="I7" s="15">
+        <f>SUM(I4:I6)</f>
+        <v/>
+      </c>
+      <c r="J7" s="15">
+        <f>SUM(J4:J6)</f>
+        <v/>
+      </c>
+      <c r="K7" s="15">
+        <f>SUM(K4:K6)</f>
+        <v/>
+      </c>
+      <c r="L7" s="15">
+        <f>SUM(L4:L6)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n"/>
-      <c r="B9" s="13" t="n"/>
-      <c r="C9" s="13" t="n"/>
-      <c r="D9" s="13" t="n"/>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="13" t="n"/>
-      <c r="G9" s="13" t="n"/>
-      <c r="H9" s="13" t="n"/>
-      <c r="I9" s="13" t="n"/>
-      <c r="J9" s="13" t="n"/>
-      <c r="K9" s="13" t="n"/>
-      <c r="L9" s="11">
-        <f>SUM(B9:K9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="13" t="n"/>
-      <c r="C10" s="13" t="n"/>
-      <c r="D10" s="13" t="n"/>
-      <c r="E10" s="13" t="n"/>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n"/>
-      <c r="I10" s="13" t="n"/>
-      <c r="J10" s="13" t="n"/>
-      <c r="K10" s="13" t="n"/>
-      <c r="L10" s="11">
-        <f>SUM(B10:K10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="n"/>
-      <c r="B11" s="13" t="n"/>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="13" t="n"/>
-      <c r="H11" s="13" t="n"/>
-      <c r="I11" s="13" t="n"/>
-      <c r="J11" s="13" t="n"/>
-      <c r="K11" s="13" t="n"/>
-      <c r="L11" s="11">
-        <f>SUM(B11:K11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="13" t="n"/>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="13" t="n"/>
-      <c r="G12" s="13" t="n"/>
-      <c r="H12" s="13" t="n"/>
-      <c r="I12" s="13" t="n"/>
-      <c r="J12" s="13" t="n"/>
-      <c r="K12" s="13" t="n"/>
-      <c r="L12" s="11">
-        <f>SUM(B12:K12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="n"/>
-      <c r="B13" s="13" t="n"/>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="13" t="n"/>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="13" t="n"/>
-      <c r="G13" s="13" t="n"/>
-      <c r="H13" s="13" t="n"/>
-      <c r="I13" s="13" t="n"/>
-      <c r="J13" s="13" t="n"/>
-      <c r="K13" s="13" t="n"/>
-      <c r="L13" s="11">
-        <f>SUM(B13:K13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="13" t="n"/>
-      <c r="C14" s="13" t="n"/>
-      <c r="D14" s="13" t="n"/>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="13" t="n"/>
-      <c r="G14" s="13" t="n"/>
-      <c r="H14" s="13" t="n"/>
-      <c r="I14" s="13" t="n"/>
-      <c r="J14" s="13" t="n"/>
-      <c r="K14" s="13" t="n"/>
-      <c r="L14" s="11">
-        <f>SUM(B14:K14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="B15" s="13" t="n"/>
-      <c r="C15" s="13" t="n"/>
-      <c r="D15" s="13" t="n"/>
-      <c r="E15" s="13" t="n"/>
-      <c r="F15" s="13" t="n"/>
-      <c r="G15" s="13" t="n"/>
-      <c r="H15" s="13" t="n"/>
-      <c r="I15" s="13" t="n"/>
-      <c r="J15" s="13" t="n"/>
-      <c r="K15" s="13" t="n"/>
-      <c r="L15" s="11">
-        <f>SUM(B15:K15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="13" t="n"/>
-      <c r="C16" s="13" t="n"/>
-      <c r="D16" s="13" t="n"/>
-      <c r="E16" s="13" t="n"/>
-      <c r="F16" s="13" t="n"/>
-      <c r="G16" s="13" t="n"/>
-      <c r="H16" s="13" t="n"/>
-      <c r="I16" s="13" t="n"/>
-      <c r="J16" s="13" t="n"/>
-      <c r="K16" s="13" t="n"/>
-      <c r="L16" s="11">
-        <f>SUM(B16:K16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="B17" s="13" t="n"/>
-      <c r="C17" s="13" t="n"/>
-      <c r="D17" s="13" t="n"/>
-      <c r="E17" s="13" t="n"/>
-      <c r="F17" s="13" t="n"/>
-      <c r="G17" s="13" t="n"/>
-      <c r="H17" s="13" t="n"/>
-      <c r="I17" s="13" t="n"/>
-      <c r="J17" s="13" t="n"/>
-      <c r="K17" s="13" t="n"/>
-      <c r="L17" s="11">
-        <f>SUM(B17:K17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="13" t="n"/>
-      <c r="C18" s="13" t="n"/>
-      <c r="D18" s="13" t="n"/>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="13" t="n"/>
-      <c r="G18" s="13" t="n"/>
-      <c r="H18" s="13" t="n"/>
-      <c r="I18" s="13" t="n"/>
-      <c r="J18" s="13" t="n"/>
-      <c r="K18" s="13" t="n"/>
-      <c r="L18" s="11">
-        <f>SUM(B18:K18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="n"/>
-      <c r="B19" s="13" t="n"/>
-      <c r="C19" s="13" t="n"/>
-      <c r="D19" s="13" t="n"/>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="13" t="n"/>
-      <c r="G19" s="13" t="n"/>
-      <c r="H19" s="13" t="n"/>
-      <c r="I19" s="13" t="n"/>
-      <c r="J19" s="13" t="n"/>
-      <c r="K19" s="13" t="n"/>
-      <c r="L19" s="11">
-        <f>SUM(B19:K19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="13" t="n"/>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="13" t="n"/>
-      <c r="G20" s="13" t="n"/>
-      <c r="H20" s="13" t="n"/>
-      <c r="I20" s="13" t="n"/>
-      <c r="J20" s="13" t="n"/>
-      <c r="K20" s="13" t="n"/>
-      <c r="L20" s="11">
-        <f>SUM(B20:K20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="12" t="n"/>
-      <c r="B21" s="13" t="n"/>
-      <c r="C21" s="13" t="n"/>
-      <c r="D21" s="13" t="n"/>
-      <c r="E21" s="13" t="n"/>
-      <c r="F21" s="13" t="n"/>
-      <c r="G21" s="13" t="n"/>
-      <c r="H21" s="13" t="n"/>
-      <c r="I21" s="13" t="n"/>
-      <c r="J21" s="13" t="n"/>
-      <c r="K21" s="13" t="n"/>
-      <c r="L21" s="11">
-        <f>SUM(B21:K21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="13" t="n"/>
-      <c r="C22" s="13" t="n"/>
-      <c r="D22" s="13" t="n"/>
-      <c r="E22" s="13" t="n"/>
-      <c r="F22" s="13" t="n"/>
-      <c r="G22" s="13" t="n"/>
-      <c r="H22" s="13" t="n"/>
-      <c r="I22" s="13" t="n"/>
-      <c r="J22" s="13" t="n"/>
-      <c r="K22" s="13" t="n"/>
-      <c r="L22" s="11">
-        <f>SUM(B22:K22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="12" t="n"/>
-      <c r="B23" s="13" t="n"/>
-      <c r="C23" s="13" t="n"/>
-      <c r="D23" s="13" t="n"/>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="13" t="n"/>
-      <c r="G23" s="13" t="n"/>
-      <c r="H23" s="13" t="n"/>
-      <c r="I23" s="13" t="n"/>
-      <c r="J23" s="13" t="n"/>
-      <c r="K23" s="13" t="n"/>
-      <c r="L23" s="11">
-        <f>SUM(B23:K23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="12" t="n"/>
-      <c r="B24" s="13" t="n"/>
-      <c r="C24" s="13" t="n"/>
-      <c r="D24" s="13" t="n"/>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="13" t="n"/>
-      <c r="G24" s="13" t="n"/>
-      <c r="H24" s="13" t="n"/>
-      <c r="I24" s="13" t="n"/>
-      <c r="J24" s="13" t="n"/>
-      <c r="K24" s="13" t="n"/>
-      <c r="L24" s="11">
-        <f>SUM(B24:K24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="12" t="n"/>
-      <c r="B25" s="13" t="n"/>
-      <c r="C25" s="13" t="n"/>
-      <c r="D25" s="13" t="n"/>
-      <c r="E25" s="13" t="n"/>
-      <c r="F25" s="13" t="n"/>
-      <c r="G25" s="13" t="n"/>
-      <c r="H25" s="13" t="n"/>
-      <c r="I25" s="13" t="n"/>
-      <c r="J25" s="13" t="n"/>
-      <c r="K25" s="13" t="n"/>
-      <c r="L25" s="11">
-        <f>SUM(B25:K25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="n"/>
-      <c r="B26" s="13" t="n"/>
-      <c r="C26" s="13" t="n"/>
-      <c r="D26" s="13" t="n"/>
-      <c r="E26" s="13" t="n"/>
-      <c r="F26" s="13" t="n"/>
-      <c r="G26" s="13" t="n"/>
-      <c r="H26" s="13" t="n"/>
-      <c r="I26" s="13" t="n"/>
-      <c r="J26" s="13" t="n"/>
-      <c r="K26" s="13" t="n"/>
-      <c r="L26" s="11">
-        <f>SUM(B26:K26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="n"/>
-      <c r="B27" s="13" t="n"/>
-      <c r="C27" s="13" t="n"/>
-      <c r="D27" s="13" t="n"/>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="13" t="n"/>
-      <c r="G27" s="13" t="n"/>
-      <c r="H27" s="13" t="n"/>
-      <c r="I27" s="13" t="n"/>
-      <c r="J27" s="13" t="n"/>
-      <c r="K27" s="13" t="n"/>
-      <c r="L27" s="11">
-        <f>SUM(B27:K27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="12" t="n"/>
-      <c r="B28" s="13" t="n"/>
-      <c r="C28" s="13" t="n"/>
-      <c r="D28" s="13" t="n"/>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="13" t="n"/>
-      <c r="G28" s="13" t="n"/>
-      <c r="H28" s="13" t="n"/>
-      <c r="I28" s="13" t="n"/>
-      <c r="J28" s="13" t="n"/>
-      <c r="K28" s="13" t="n"/>
-      <c r="L28" s="11">
-        <f>SUM(B28:K28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="12" t="n"/>
-      <c r="B29" s="13" t="n"/>
-      <c r="C29" s="13" t="n"/>
-      <c r="D29" s="13" t="n"/>
-      <c r="E29" s="13" t="n"/>
-      <c r="F29" s="13" t="n"/>
-      <c r="G29" s="13" t="n"/>
-      <c r="H29" s="13" t="n"/>
-      <c r="I29" s="13" t="n"/>
-      <c r="J29" s="13" t="n"/>
-      <c r="K29" s="13" t="n"/>
-      <c r="L29" s="11">
-        <f>SUM(B29:K29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="n"/>
-      <c r="B30" s="13" t="n"/>
-      <c r="C30" s="13" t="n"/>
-      <c r="D30" s="13" t="n"/>
-      <c r="E30" s="13" t="n"/>
-      <c r="F30" s="13" t="n"/>
-      <c r="G30" s="13" t="n"/>
-      <c r="H30" s="13" t="n"/>
-      <c r="I30" s="13" t="n"/>
-      <c r="J30" s="13" t="n"/>
-      <c r="K30" s="13" t="n"/>
-      <c r="L30" s="11">
-        <f>SUM(B30:K30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="12" t="n"/>
-      <c r="B31" s="13" t="n"/>
-      <c r="C31" s="13" t="n"/>
-      <c r="D31" s="13" t="n"/>
-      <c r="E31" s="13" t="n"/>
-      <c r="F31" s="13" t="n"/>
-      <c r="G31" s="13" t="n"/>
-      <c r="H31" s="13" t="n"/>
-      <c r="I31" s="13" t="n"/>
-      <c r="J31" s="13" t="n"/>
-      <c r="K31" s="13" t="n"/>
-      <c r="L31" s="11">
-        <f>SUM(B31:K31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="12" t="n"/>
-      <c r="B32" s="13" t="n"/>
-      <c r="C32" s="13" t="n"/>
-      <c r="D32" s="13" t="n"/>
-      <c r="E32" s="13" t="n"/>
-      <c r="F32" s="13" t="n"/>
-      <c r="G32" s="13" t="n"/>
-      <c r="H32" s="13" t="n"/>
-      <c r="I32" s="13" t="n"/>
-      <c r="J32" s="13" t="n"/>
-      <c r="K32" s="13" t="n"/>
-      <c r="L32" s="11">
-        <f>SUM(B32:K32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="12" t="n"/>
-      <c r="B33" s="13" t="n"/>
-      <c r="C33" s="13" t="n"/>
-      <c r="D33" s="13" t="n"/>
-      <c r="E33" s="13" t="n"/>
-      <c r="F33" s="13" t="n"/>
-      <c r="G33" s="13" t="n"/>
-      <c r="H33" s="13" t="n"/>
-      <c r="I33" s="13" t="n"/>
-      <c r="J33" s="13" t="n"/>
-      <c r="K33" s="13" t="n"/>
-      <c r="L33" s="11">
-        <f>SUM(B33:K33)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="12" t="n"/>
-      <c r="B34" s="13" t="n"/>
-      <c r="C34" s="13" t="n"/>
-      <c r="D34" s="13" t="n"/>
-      <c r="E34" s="13" t="n"/>
-      <c r="F34" s="13" t="n"/>
-      <c r="G34" s="13" t="n"/>
-      <c r="H34" s="13" t="n"/>
-      <c r="I34" s="13" t="n"/>
-      <c r="J34" s="13" t="n"/>
-      <c r="K34" s="13" t="n"/>
-      <c r="L34" s="11">
-        <f>SUM(B34:K34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="n"/>
-      <c r="B35" s="13" t="n"/>
-      <c r="C35" s="13" t="n"/>
-      <c r="D35" s="13" t="n"/>
-      <c r="E35" s="13" t="n"/>
-      <c r="F35" s="13" t="n"/>
-      <c r="G35" s="13" t="n"/>
-      <c r="H35" s="13" t="n"/>
-      <c r="I35" s="13" t="n"/>
-      <c r="J35" s="13" t="n"/>
-      <c r="K35" s="13" t="n"/>
-      <c r="L35" s="11">
-        <f>SUM(B35:K35)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="12" t="n"/>
-      <c r="B36" s="13" t="n"/>
-      <c r="C36" s="13" t="n"/>
-      <c r="D36" s="13" t="n"/>
-      <c r="E36" s="13" t="n"/>
-      <c r="F36" s="13" t="n"/>
-      <c r="G36" s="13" t="n"/>
-      <c r="H36" s="13" t="n"/>
-      <c r="I36" s="13" t="n"/>
-      <c r="J36" s="13" t="n"/>
-      <c r="K36" s="13" t="n"/>
-      <c r="L36" s="11">
-        <f>SUM(B36:K36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="12" t="n"/>
-      <c r="B37" s="13" t="n"/>
-      <c r="C37" s="13" t="n"/>
-      <c r="D37" s="13" t="n"/>
-      <c r="E37" s="13" t="n"/>
-      <c r="F37" s="13" t="n"/>
-      <c r="G37" s="13" t="n"/>
-      <c r="H37" s="13" t="n"/>
-      <c r="I37" s="13" t="n"/>
-      <c r="J37" s="13" t="n"/>
-      <c r="K37" s="13" t="n"/>
-      <c r="L37" s="11">
-        <f>SUM(B37:K37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="14" t="inlineStr">
-        <is>
-          <t>TOTAL GENERAL</t>
-        </is>
-      </c>
-      <c r="B38" s="15">
-        <f>SUM(B8:B37)</f>
-        <v/>
-      </c>
-      <c r="C38" s="15">
-        <f>SUM(C8:C37)</f>
-        <v/>
-      </c>
-      <c r="D38" s="15">
-        <f>SUM(D8:D37)</f>
-        <v/>
-      </c>
-      <c r="E38" s="15">
-        <f>SUM(E8:E37)</f>
-        <v/>
-      </c>
-      <c r="F38" s="15">
-        <f>SUM(F8:F37)</f>
-        <v/>
-      </c>
-      <c r="G38" s="15">
-        <f>SUM(G8:G37)</f>
-        <v/>
-      </c>
-      <c r="H38" s="15">
-        <f>SUM(H8:H37)</f>
-        <v/>
-      </c>
-      <c r="I38" s="15">
-        <f>SUM(I8:I37)</f>
-        <v/>
-      </c>
-      <c r="J38" s="15">
-        <f>SUM(J8:J37)</f>
-        <v/>
-      </c>
-      <c r="K38" s="15">
-        <f>SUM(K8:K37)</f>
-        <v/>
-      </c>
-      <c r="L38" s="15">
-        <f>SUM(L8:L37)</f>
-        <v/>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Este valor de TOTAL GENERAL (columna L) es el que se digita en el sistema.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="J6:J7"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A4:L4"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="L6:L7"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="G2:L2"/>
-    <mergeCell ref="I3:L3"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="K6:K7"/>
+  <mergeCells count="2">
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1307,6 +945,17 @@
           <t>JORNADA DE VACUNACION 2026</t>
         </is>
       </c>
+      <c r="B1" s="18" t="n"/>
+      <c r="C1" s="18" t="n"/>
+      <c r="D1" s="18" t="n"/>
+      <c r="E1" s="18" t="n"/>
+      <c r="F1" s="18" t="n"/>
+      <c r="G1" s="18" t="n"/>
+      <c r="H1" s="18" t="n"/>
+      <c r="I1" s="18" t="n"/>
+      <c r="J1" s="18" t="n"/>
+      <c r="K1" s="18" t="n"/>
+      <c r="L1" s="19" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1314,18 +963,25 @@
           <t>FECHA:</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
       <c r="C2" s="3" t="n"/>
-      <c r="D2" s="4" t="n"/>
+      <c r="D2" s="19" t="n"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>NOMBRES DEL RESPONSABLE:</t>
         </is>
       </c>
+      <c r="F2" s="19" t="n"/>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Mónica</t>
-        </is>
-      </c>
+          <t>Yesenia</t>
+        </is>
+      </c>
+      <c r="H2" s="18" t="n"/>
+      <c r="I2" s="18" t="n"/>
+      <c r="J2" s="18" t="n"/>
+      <c r="K2" s="18" t="n"/>
+      <c r="L2" s="19" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -1333,16 +989,25 @@
           <t>RENIPRESS: 00006126</t>
         </is>
       </c>
+      <c r="B3" s="18" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>EESS: PS. PRINCIPE DE ASTURIAS</t>
         </is>
       </c>
+      <c r="E3" s="18" t="n"/>
+      <c r="F3" s="18" t="n"/>
+      <c r="G3" s="18" t="n"/>
+      <c r="H3" s="19" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>RIS: RIS VILLA EL SALVADOR</t>
         </is>
       </c>
+      <c r="J3" s="18" t="n"/>
+      <c r="K3" s="18" t="n"/>
+      <c r="L3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1368,11 +1033,13 @@
           <t>NIÑOS 1 AÑO</t>
         </is>
       </c>
+      <c r="D6" s="19" t="n"/>
       <c r="E6" s="7" t="inlineStr">
         <is>
           <t>NIÑOS 2 - 4 AÑOS</t>
         </is>
       </c>
+      <c r="F6" s="19" t="n"/>
       <c r="G6" s="7" t="inlineStr">
         <is>
           <t>5 - 10 AÑOS
@@ -1409,6 +1076,8 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="20" t="n"/>
+      <c r="B7" s="20" t="n"/>
       <c r="C7" s="8" t="inlineStr">
         <is>
           <t>SPR 1RA</t>
@@ -1429,6 +1098,12 @@
           <t>SPR 2DA</t>
         </is>
       </c>
+      <c r="G7" s="20" t="n"/>
+      <c r="H7" s="20" t="n"/>
+      <c r="I7" s="20" t="n"/>
+      <c r="J7" s="20" t="n"/>
+      <c r="K7" s="20" t="n"/>
+      <c r="L7" s="20" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n">
@@ -2068,6 +1743,17 @@
           <t>JORNADA DE VACUNACION 2026</t>
         </is>
       </c>
+      <c r="B1" s="18" t="n"/>
+      <c r="C1" s="18" t="n"/>
+      <c r="D1" s="18" t="n"/>
+      <c r="E1" s="18" t="n"/>
+      <c r="F1" s="18" t="n"/>
+      <c r="G1" s="18" t="n"/>
+      <c r="H1" s="18" t="n"/>
+      <c r="I1" s="18" t="n"/>
+      <c r="J1" s="18" t="n"/>
+      <c r="K1" s="18" t="n"/>
+      <c r="L1" s="19" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -2075,18 +1761,25 @@
           <t>FECHA:</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
       <c r="C2" s="3" t="n"/>
-      <c r="D2" s="4" t="n"/>
+      <c r="D2" s="19" t="n"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>NOMBRES DEL RESPONSABLE:</t>
         </is>
       </c>
+      <c r="F2" s="19" t="n"/>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Cirila</t>
-        </is>
-      </c>
+          <t>Mónica</t>
+        </is>
+      </c>
+      <c r="H2" s="18" t="n"/>
+      <c r="I2" s="18" t="n"/>
+      <c r="J2" s="18" t="n"/>
+      <c r="K2" s="18" t="n"/>
+      <c r="L2" s="19" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -2094,16 +1787,25 @@
           <t>RENIPRESS: 00006126</t>
         </is>
       </c>
+      <c r="B3" s="18" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>EESS: PS. PRINCIPE DE ASTURIAS</t>
         </is>
       </c>
+      <c r="E3" s="18" t="n"/>
+      <c r="F3" s="18" t="n"/>
+      <c r="G3" s="18" t="n"/>
+      <c r="H3" s="19" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>RIS: RIS VILLA EL SALVADOR</t>
         </is>
       </c>
+      <c r="J3" s="18" t="n"/>
+      <c r="K3" s="18" t="n"/>
+      <c r="L3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2129,11 +1831,13 @@
           <t>NIÑOS 1 AÑO</t>
         </is>
       </c>
+      <c r="D6" s="19" t="n"/>
       <c r="E6" s="7" t="inlineStr">
         <is>
           <t>NIÑOS 2 - 4 AÑOS</t>
         </is>
       </c>
+      <c r="F6" s="19" t="n"/>
       <c r="G6" s="7" t="inlineStr">
         <is>
           <t>5 - 10 AÑOS
@@ -2170,6 +1874,8 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="20" t="n"/>
+      <c r="B7" s="20" t="n"/>
       <c r="C7" s="8" t="inlineStr">
         <is>
           <t>SPR 1RA</t>
@@ -2190,6 +1896,810 @@
           <t>SPR 2DA</t>
         </is>
       </c>
+      <c r="G7" s="20" t="n"/>
+      <c r="H7" s="20" t="n"/>
+      <c r="I7" s="20" t="n"/>
+      <c r="J7" s="20" t="n"/>
+      <c r="K7" s="20" t="n"/>
+      <c r="L7" s="20" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="11">
+        <f>SUM(B8:K8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n"/>
+      <c r="B9" s="13" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="13" t="n"/>
+      <c r="F9" s="13" t="n"/>
+      <c r="G9" s="13" t="n"/>
+      <c r="H9" s="13" t="n"/>
+      <c r="I9" s="13" t="n"/>
+      <c r="J9" s="13" t="n"/>
+      <c r="K9" s="13" t="n"/>
+      <c r="L9" s="11">
+        <f>SUM(B9:K9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="13" t="n"/>
+      <c r="C10" s="13" t="n"/>
+      <c r="D10" s="13" t="n"/>
+      <c r="E10" s="13" t="n"/>
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="13" t="n"/>
+      <c r="H10" s="13" t="n"/>
+      <c r="I10" s="13" t="n"/>
+      <c r="J10" s="13" t="n"/>
+      <c r="K10" s="13" t="n"/>
+      <c r="L10" s="11">
+        <f>SUM(B10:K10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="13" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="13" t="n"/>
+      <c r="F11" s="13" t="n"/>
+      <c r="G11" s="13" t="n"/>
+      <c r="H11" s="13" t="n"/>
+      <c r="I11" s="13" t="n"/>
+      <c r="J11" s="13" t="n"/>
+      <c r="K11" s="13" t="n"/>
+      <c r="L11" s="11">
+        <f>SUM(B11:K11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="13" t="n"/>
+      <c r="I12" s="13" t="n"/>
+      <c r="J12" s="13" t="n"/>
+      <c r="K12" s="13" t="n"/>
+      <c r="L12" s="11">
+        <f>SUM(B12:K12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+      <c r="H13" s="13" t="n"/>
+      <c r="I13" s="13" t="n"/>
+      <c r="J13" s="13" t="n"/>
+      <c r="K13" s="13" t="n"/>
+      <c r="L13" s="11">
+        <f>SUM(B13:K13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="13" t="n"/>
+      <c r="I14" s="13" t="n"/>
+      <c r="J14" s="13" t="n"/>
+      <c r="K14" s="13" t="n"/>
+      <c r="L14" s="11">
+        <f>SUM(B14:K14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="13" t="n"/>
+      <c r="C15" s="13" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="13" t="n"/>
+      <c r="G15" s="13" t="n"/>
+      <c r="H15" s="13" t="n"/>
+      <c r="I15" s="13" t="n"/>
+      <c r="J15" s="13" t="n"/>
+      <c r="K15" s="13" t="n"/>
+      <c r="L15" s="11">
+        <f>SUM(B15:K15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="13" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="13" t="n"/>
+      <c r="I16" s="13" t="n"/>
+      <c r="J16" s="13" t="n"/>
+      <c r="K16" s="13" t="n"/>
+      <c r="L16" s="11">
+        <f>SUM(B16:K16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="13" t="n"/>
+      <c r="F17" s="13" t="n"/>
+      <c r="G17" s="13" t="n"/>
+      <c r="H17" s="13" t="n"/>
+      <c r="I17" s="13" t="n"/>
+      <c r="J17" s="13" t="n"/>
+      <c r="K17" s="13" t="n"/>
+      <c r="L17" s="11">
+        <f>SUM(B17:K17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="13" t="n"/>
+      <c r="I18" s="13" t="n"/>
+      <c r="J18" s="13" t="n"/>
+      <c r="K18" s="13" t="n"/>
+      <c r="L18" s="11">
+        <f>SUM(B18:K18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="n"/>
+      <c r="K19" s="13" t="n"/>
+      <c r="L19" s="11">
+        <f>SUM(B19:K19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="13" t="n"/>
+      <c r="D20" s="13" t="n"/>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="13" t="n"/>
+      <c r="G20" s="13" t="n"/>
+      <c r="H20" s="13" t="n"/>
+      <c r="I20" s="13" t="n"/>
+      <c r="J20" s="13" t="n"/>
+      <c r="K20" s="13" t="n"/>
+      <c r="L20" s="11">
+        <f>SUM(B20:K20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n"/>
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="13" t="n"/>
+      <c r="D21" s="13" t="n"/>
+      <c r="E21" s="13" t="n"/>
+      <c r="F21" s="13" t="n"/>
+      <c r="G21" s="13" t="n"/>
+      <c r="H21" s="13" t="n"/>
+      <c r="I21" s="13" t="n"/>
+      <c r="J21" s="13" t="n"/>
+      <c r="K21" s="13" t="n"/>
+      <c r="L21" s="11">
+        <f>SUM(B21:K21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n"/>
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="n"/>
+      <c r="D22" s="13" t="n"/>
+      <c r="E22" s="13" t="n"/>
+      <c r="F22" s="13" t="n"/>
+      <c r="G22" s="13" t="n"/>
+      <c r="H22" s="13" t="n"/>
+      <c r="I22" s="13" t="n"/>
+      <c r="J22" s="13" t="n"/>
+      <c r="K22" s="13" t="n"/>
+      <c r="L22" s="11">
+        <f>SUM(B22:K22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n"/>
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="n"/>
+      <c r="D23" s="13" t="n"/>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="13" t="n"/>
+      <c r="G23" s="13" t="n"/>
+      <c r="H23" s="13" t="n"/>
+      <c r="I23" s="13" t="n"/>
+      <c r="J23" s="13" t="n"/>
+      <c r="K23" s="13" t="n"/>
+      <c r="L23" s="11">
+        <f>SUM(B23:K23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n"/>
+      <c r="B24" s="13" t="n"/>
+      <c r="C24" s="13" t="n"/>
+      <c r="D24" s="13" t="n"/>
+      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="13" t="n"/>
+      <c r="G24" s="13" t="n"/>
+      <c r="H24" s="13" t="n"/>
+      <c r="I24" s="13" t="n"/>
+      <c r="J24" s="13" t="n"/>
+      <c r="K24" s="13" t="n"/>
+      <c r="L24" s="11">
+        <f>SUM(B24:K24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n"/>
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="13" t="n"/>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="13" t="n"/>
+      <c r="F25" s="13" t="n"/>
+      <c r="G25" s="13" t="n"/>
+      <c r="H25" s="13" t="n"/>
+      <c r="I25" s="13" t="n"/>
+      <c r="J25" s="13" t="n"/>
+      <c r="K25" s="13" t="n"/>
+      <c r="L25" s="11">
+        <f>SUM(B25:K25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n"/>
+      <c r="B26" s="13" t="n"/>
+      <c r="C26" s="13" t="n"/>
+      <c r="D26" s="13" t="n"/>
+      <c r="E26" s="13" t="n"/>
+      <c r="F26" s="13" t="n"/>
+      <c r="G26" s="13" t="n"/>
+      <c r="H26" s="13" t="n"/>
+      <c r="I26" s="13" t="n"/>
+      <c r="J26" s="13" t="n"/>
+      <c r="K26" s="13" t="n"/>
+      <c r="L26" s="11">
+        <f>SUM(B26:K26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n"/>
+      <c r="B27" s="13" t="n"/>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="13" t="n"/>
+      <c r="E27" s="13" t="n"/>
+      <c r="F27" s="13" t="n"/>
+      <c r="G27" s="13" t="n"/>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="n"/>
+      <c r="J27" s="13" t="n"/>
+      <c r="K27" s="13" t="n"/>
+      <c r="L27" s="11">
+        <f>SUM(B27:K27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n"/>
+      <c r="B28" s="13" t="n"/>
+      <c r="C28" s="13" t="n"/>
+      <c r="D28" s="13" t="n"/>
+      <c r="E28" s="13" t="n"/>
+      <c r="F28" s="13" t="n"/>
+      <c r="G28" s="13" t="n"/>
+      <c r="H28" s="13" t="n"/>
+      <c r="I28" s="13" t="n"/>
+      <c r="J28" s="13" t="n"/>
+      <c r="K28" s="13" t="n"/>
+      <c r="L28" s="11">
+        <f>SUM(B28:K28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n"/>
+      <c r="B29" s="13" t="n"/>
+      <c r="C29" s="13" t="n"/>
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="13" t="n"/>
+      <c r="F29" s="13" t="n"/>
+      <c r="G29" s="13" t="n"/>
+      <c r="H29" s="13" t="n"/>
+      <c r="I29" s="13" t="n"/>
+      <c r="J29" s="13" t="n"/>
+      <c r="K29" s="13" t="n"/>
+      <c r="L29" s="11">
+        <f>SUM(B29:K29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n"/>
+      <c r="B30" s="13" t="n"/>
+      <c r="C30" s="13" t="n"/>
+      <c r="D30" s="13" t="n"/>
+      <c r="E30" s="13" t="n"/>
+      <c r="F30" s="13" t="n"/>
+      <c r="G30" s="13" t="n"/>
+      <c r="H30" s="13" t="n"/>
+      <c r="I30" s="13" t="n"/>
+      <c r="J30" s="13" t="n"/>
+      <c r="K30" s="13" t="n"/>
+      <c r="L30" s="11">
+        <f>SUM(B30:K30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n"/>
+      <c r="B31" s="13" t="n"/>
+      <c r="C31" s="13" t="n"/>
+      <c r="D31" s="13" t="n"/>
+      <c r="E31" s="13" t="n"/>
+      <c r="F31" s="13" t="n"/>
+      <c r="G31" s="13" t="n"/>
+      <c r="H31" s="13" t="n"/>
+      <c r="I31" s="13" t="n"/>
+      <c r="J31" s="13" t="n"/>
+      <c r="K31" s="13" t="n"/>
+      <c r="L31" s="11">
+        <f>SUM(B31:K31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n"/>
+      <c r="B32" s="13" t="n"/>
+      <c r="C32" s="13" t="n"/>
+      <c r="D32" s="13" t="n"/>
+      <c r="E32" s="13" t="n"/>
+      <c r="F32" s="13" t="n"/>
+      <c r="G32" s="13" t="n"/>
+      <c r="H32" s="13" t="n"/>
+      <c r="I32" s="13" t="n"/>
+      <c r="J32" s="13" t="n"/>
+      <c r="K32" s="13" t="n"/>
+      <c r="L32" s="11">
+        <f>SUM(B32:K32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n"/>
+      <c r="B33" s="13" t="n"/>
+      <c r="C33" s="13" t="n"/>
+      <c r="D33" s="13" t="n"/>
+      <c r="E33" s="13" t="n"/>
+      <c r="F33" s="13" t="n"/>
+      <c r="G33" s="13" t="n"/>
+      <c r="H33" s="13" t="n"/>
+      <c r="I33" s="13" t="n"/>
+      <c r="J33" s="13" t="n"/>
+      <c r="K33" s="13" t="n"/>
+      <c r="L33" s="11">
+        <f>SUM(B33:K33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="n"/>
+      <c r="B34" s="13" t="n"/>
+      <c r="C34" s="13" t="n"/>
+      <c r="D34" s="13" t="n"/>
+      <c r="E34" s="13" t="n"/>
+      <c r="F34" s="13" t="n"/>
+      <c r="G34" s="13" t="n"/>
+      <c r="H34" s="13" t="n"/>
+      <c r="I34" s="13" t="n"/>
+      <c r="J34" s="13" t="n"/>
+      <c r="K34" s="13" t="n"/>
+      <c r="L34" s="11">
+        <f>SUM(B34:K34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n"/>
+      <c r="B35" s="13" t="n"/>
+      <c r="C35" s="13" t="n"/>
+      <c r="D35" s="13" t="n"/>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="13" t="n"/>
+      <c r="G35" s="13" t="n"/>
+      <c r="H35" s="13" t="n"/>
+      <c r="I35" s="13" t="n"/>
+      <c r="J35" s="13" t="n"/>
+      <c r="K35" s="13" t="n"/>
+      <c r="L35" s="11">
+        <f>SUM(B35:K35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n"/>
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="13" t="n"/>
+      <c r="D36" s="13" t="n"/>
+      <c r="E36" s="13" t="n"/>
+      <c r="F36" s="13" t="n"/>
+      <c r="G36" s="13" t="n"/>
+      <c r="H36" s="13" t="n"/>
+      <c r="I36" s="13" t="n"/>
+      <c r="J36" s="13" t="n"/>
+      <c r="K36" s="13" t="n"/>
+      <c r="L36" s="11">
+        <f>SUM(B36:K36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n"/>
+      <c r="B37" s="13" t="n"/>
+      <c r="C37" s="13" t="n"/>
+      <c r="D37" s="13" t="n"/>
+      <c r="E37" s="13" t="n"/>
+      <c r="F37" s="13" t="n"/>
+      <c r="G37" s="13" t="n"/>
+      <c r="H37" s="13" t="n"/>
+      <c r="I37" s="13" t="n"/>
+      <c r="J37" s="13" t="n"/>
+      <c r="K37" s="13" t="n"/>
+      <c r="L37" s="11">
+        <f>SUM(B37:K37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B38" s="15">
+        <f>SUM(B8:B37)</f>
+        <v/>
+      </c>
+      <c r="C38" s="15">
+        <f>SUM(C8:C37)</f>
+        <v/>
+      </c>
+      <c r="D38" s="15">
+        <f>SUM(D8:D37)</f>
+        <v/>
+      </c>
+      <c r="E38" s="15">
+        <f>SUM(E8:E37)</f>
+        <v/>
+      </c>
+      <c r="F38" s="15">
+        <f>SUM(F8:F37)</f>
+        <v/>
+      </c>
+      <c r="G38" s="15">
+        <f>SUM(G8:G37)</f>
+        <v/>
+      </c>
+      <c r="H38" s="15">
+        <f>SUM(H8:H37)</f>
+        <v/>
+      </c>
+      <c r="I38" s="15">
+        <f>SUM(I8:I37)</f>
+        <v/>
+      </c>
+      <c r="J38" s="15">
+        <f>SUM(J8:J37)</f>
+        <v/>
+      </c>
+      <c r="K38" s="15">
+        <f>SUM(K8:K37)</f>
+        <v/>
+      </c>
+      <c r="L38" s="15">
+        <f>SUM(L8:L37)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="G2:L2"/>
+    <mergeCell ref="I3:L3"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="K6:K7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>JORNADA DE VACUNACION 2026</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="n"/>
+      <c r="C1" s="18" t="n"/>
+      <c r="D1" s="18" t="n"/>
+      <c r="E1" s="18" t="n"/>
+      <c r="F1" s="18" t="n"/>
+      <c r="G1" s="18" t="n"/>
+      <c r="H1" s="18" t="n"/>
+      <c r="I1" s="18" t="n"/>
+      <c r="J1" s="18" t="n"/>
+      <c r="K1" s="18" t="n"/>
+      <c r="L1" s="19" t="n"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>FECHA:</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="19" t="n"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>NOMBRES DEL RESPONSABLE:</t>
+        </is>
+      </c>
+      <c r="F2" s="19" t="n"/>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Cirila</t>
+        </is>
+      </c>
+      <c r="H2" s="18" t="n"/>
+      <c r="I2" s="18" t="n"/>
+      <c r="J2" s="18" t="n"/>
+      <c r="K2" s="18" t="n"/>
+      <c r="L2" s="19" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>RENIPRESS: 00006126</t>
+        </is>
+      </c>
+      <c r="B3" s="18" t="n"/>
+      <c r="C3" s="19" t="n"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>EESS: PS. PRINCIPE DE ASTURIAS</t>
+        </is>
+      </c>
+      <c r="E3" s="18" t="n"/>
+      <c r="F3" s="18" t="n"/>
+      <c r="G3" s="18" t="n"/>
+      <c r="H3" s="19" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>RIS: RIS VILLA EL SALVADOR</t>
+        </is>
+      </c>
+      <c r="J3" s="18" t="n"/>
+      <c r="K3" s="18" t="n"/>
+      <c r="L3" s="19" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Leyenda: complete FECHA por cada jornada; use "-" o deje en blanco cuando no se aplican dosis de ese indicador. La columna TOTAL DOSIS se calcula automaticamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>FECHA / INDICADORES</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>MENORES DE 1 AÑO
+PENTAV 3RA</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>NIÑOS 1 AÑO</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="n"/>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>NIÑOS 2 - 4 AÑOS</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>5 - 10 AÑOS
+SPR UNICA</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>9 AÑOS
+VPH</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>GESTANTE
+DTPA</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>60 AÑOS A MAS
+NEUMO</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>OTRAS VACUNAS</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL DOSIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="20" t="n"/>
+      <c r="B7" s="20" t="n"/>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>SPR 1RA</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>SPR 2DA</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>SPR 1RA</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>SPR 2DA</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="n"/>
+      <c r="H7" s="20" t="n"/>
+      <c r="I7" s="20" t="n"/>
+      <c r="J7" s="20" t="n"/>
+      <c r="K7" s="20" t="n"/>
+      <c r="L7" s="20" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n">

</xml_diff>